<commit_message>
Removed the output box
</commit_message>
<xml_diff>
--- a/Payment Terms.xlsx
+++ b/Payment Terms.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cabinet\App Projects\Payment Terms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C53AE1-9317-49BB-ABA4-EC9E9346CDEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81606991-548D-4105-8314-C118613668A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{EB5A27B0-2CAD-424F-89DA-FF45EE1C670D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{EB5A27B0-2CAD-424F-89DA-FF45EE1C670D}"/>
   </bookViews>
   <sheets>
     <sheet name="New Payments" sheetId="1" r:id="rId1"/>
@@ -711,10 +711,10 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3172,15 +3172,15 @@
         <v>8.6199999999999999E-2</v>
       </c>
       <c r="E35" s="8">
-        <f t="shared" si="7"/>
-        <v>1120.7283263622139</v>
+        <f t="shared" ref="E35:E46" si="9">PMT(D35/12,C35,-84995,G35)</f>
+        <v>1293.4524285308762</v>
       </c>
       <c r="F35" s="9">
         <v>0.4</v>
       </c>
       <c r="G35" s="10">
-        <f t="shared" si="8"/>
-        <v>29458</v>
+        <f t="shared" ref="G35:G46" si="10">SUM(84995*F35)</f>
+        <v>33998</v>
       </c>
       <c r="H35" s="11"/>
       <c r="I35" s="12" t="s">
@@ -3231,28 +3231,28 @@
         <v>8.5300000000000001E-2</v>
       </c>
       <c r="E36" s="8">
-        <f t="shared" si="7"/>
-        <v>1034.967713218128</v>
+        <f t="shared" si="9"/>
+        <v>1194.4745846286207</v>
       </c>
       <c r="F36" s="9">
         <v>0.35</v>
       </c>
       <c r="G36" s="10">
-        <f t="shared" si="8"/>
-        <v>25775.75</v>
+        <f t="shared" si="10"/>
+        <v>29748.249999999996</v>
       </c>
       <c r="H36" s="11"/>
-      <c r="I36" s="29" t="s">
+      <c r="I36" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="J36" s="29"/>
-      <c r="K36" s="29"/>
-      <c r="L36" s="29"/>
-      <c r="M36" s="29"/>
-      <c r="N36" s="29"/>
-      <c r="O36" s="29"/>
-      <c r="P36" s="29"/>
-      <c r="Q36" s="29"/>
+      <c r="J36" s="30"/>
+      <c r="K36" s="30"/>
+      <c r="L36" s="30"/>
+      <c r="M36" s="30"/>
+      <c r="N36" s="30"/>
+      <c r="O36" s="30"/>
+      <c r="P36" s="30"/>
+      <c r="Q36" s="30"/>
       <c r="R36" s="12"/>
       <c r="S36" s="12"/>
       <c r="T36" s="12"/>
@@ -3280,15 +3280,15 @@
         <v>8.4600000000000009E-2</v>
       </c>
       <c r="E37" s="8">
-        <f t="shared" si="7"/>
-        <v>971.11719411209049</v>
+        <f t="shared" si="9"/>
+        <v>1120.7835686544524</v>
       </c>
       <c r="F37" s="9">
         <v>0.3</v>
       </c>
       <c r="G37" s="10">
-        <f t="shared" si="8"/>
-        <v>22093.5</v>
+        <f t="shared" si="10"/>
+        <v>25498.5</v>
       </c>
       <c r="H37" s="11"/>
       <c r="I37" s="20" t="s">
@@ -3339,15 +3339,15 @@
         <v>9.0499999999999997E-2</v>
       </c>
       <c r="E38" s="8">
-        <f t="shared" si="7"/>
-        <v>1679.7006572197906</v>
+        <f t="shared" si="9"/>
+        <v>1938.5723044388092</v>
       </c>
       <c r="F38" s="9">
         <v>0.6</v>
       </c>
       <c r="G38" s="10">
-        <f t="shared" si="8"/>
-        <v>44187</v>
+        <f t="shared" si="10"/>
+        <v>50997</v>
       </c>
       <c r="H38" s="11"/>
       <c r="I38" s="20" t="s">
@@ -3364,15 +3364,15 @@
         <v>6.7000000000000002E-3</v>
       </c>
       <c r="O38" s="13">
-        <f t="shared" ref="O38:Q38" si="9">$L$38*O$35</f>
+        <f t="shared" ref="O38:Q38" si="11">$L$38*O$35</f>
         <v>1.34E-2</v>
       </c>
       <c r="P38" s="13">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>2.01E-2</v>
       </c>
       <c r="Q38" s="13">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>2.6800000000000001E-2</v>
       </c>
       <c r="R38" s="12"/>
@@ -3402,15 +3402,15 @@
         <v>8.6199999999999999E-2</v>
       </c>
       <c r="E39" s="8">
-        <f t="shared" si="7"/>
-        <v>1338.9589139262678</v>
+        <f t="shared" si="9"/>
+        <v>1545.3162181976115</v>
       </c>
       <c r="F39" s="9">
         <v>0.55000000000000004</v>
       </c>
       <c r="G39" s="10">
-        <f t="shared" si="8"/>
-        <v>40504.75</v>
+        <f t="shared" si="10"/>
+        <v>46747.250000000007</v>
       </c>
       <c r="H39" s="11"/>
       <c r="I39" s="20" t="s">
@@ -3427,15 +3427,15 @@
         <v>5.1000000000000004E-3</v>
       </c>
       <c r="O39" s="13">
-        <f t="shared" ref="O39:Q39" si="10">$L$39*O$35</f>
+        <f t="shared" ref="O39:Q39" si="12">$L$39*O$35</f>
         <v>1.0200000000000001E-2</v>
       </c>
       <c r="P39" s="13">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>1.5300000000000001E-2</v>
       </c>
       <c r="Q39" s="13">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>2.0400000000000001E-2</v>
       </c>
       <c r="R39" s="12"/>
@@ -3465,15 +3465,15 @@
         <v>8.1100000000000005E-2</v>
       </c>
       <c r="E40" s="8">
-        <f t="shared" si="7"/>
-        <v>1149.7060765599892</v>
+        <f t="shared" si="9"/>
+        <v>1326.8961637207724</v>
       </c>
       <c r="F40" s="9">
         <v>0.5</v>
       </c>
       <c r="G40" s="10">
-        <f t="shared" si="8"/>
-        <v>36822.5</v>
+        <f t="shared" si="10"/>
+        <v>42497.5</v>
       </c>
       <c r="H40" s="11"/>
       <c r="I40" s="20" t="s">
@@ -3490,15 +3490,15 @@
         <v>4.1999999999999997E-3</v>
       </c>
       <c r="O40" s="13">
-        <f t="shared" ref="O40:Q40" si="11">$L$40*O$35</f>
+        <f t="shared" ref="O40:Q40" si="13">$L$40*O$35</f>
         <v>8.3999999999999995E-3</v>
       </c>
       <c r="P40" s="13">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1.26E-2</v>
       </c>
       <c r="Q40" s="13">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1.6799999999999999E-2</v>
       </c>
       <c r="R40" s="12"/>
@@ -3528,15 +3528,15 @@
         <v>8.6199999999999999E-2</v>
       </c>
       <c r="E41" s="8">
-        <f t="shared" si="7"/>
-        <v>1120.7283263622139</v>
+        <f t="shared" si="9"/>
+        <v>1293.4524285308762</v>
       </c>
       <c r="F41" s="9">
         <v>0.4</v>
       </c>
       <c r="G41" s="10">
-        <f t="shared" si="8"/>
-        <v>29458</v>
+        <f t="shared" si="10"/>
+        <v>33998</v>
       </c>
       <c r="H41" s="11"/>
       <c r="I41" s="20" t="s">
@@ -3553,15 +3553,15 @@
         <v>3.5000000000000001E-3</v>
       </c>
       <c r="O41" s="13">
-        <f t="shared" ref="O41:Q41" si="12">$L$41*O$35</f>
+        <f t="shared" ref="O41:Q41" si="14">$L$41*O$35</f>
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="P41" s="13">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>1.0500000000000001E-2</v>
       </c>
       <c r="Q41" s="13">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>1.4E-2</v>
       </c>
       <c r="R41" s="12"/>
@@ -3591,15 +3591,15 @@
         <v>8.5300000000000001E-2</v>
       </c>
       <c r="E42" s="8">
-        <f t="shared" si="7"/>
-        <v>1034.967713218128</v>
+        <f t="shared" si="9"/>
+        <v>1194.4745846286207</v>
       </c>
       <c r="F42" s="9">
         <v>0.35</v>
       </c>
       <c r="G42" s="10">
-        <f t="shared" si="8"/>
-        <v>25775.75</v>
+        <f t="shared" si="10"/>
+        <v>29748.249999999996</v>
       </c>
       <c r="H42" s="11"/>
       <c r="I42" s="20" t="s">
@@ -3616,15 +3616,15 @@
         <v>3.0999999999999999E-3</v>
       </c>
       <c r="O42" s="13">
-        <f t="shared" ref="O42:Q42" si="13">$L$42*O$35</f>
+        <f t="shared" ref="O42:Q42" si="15">$L$42*O$35</f>
         <v>6.1999999999999998E-3</v>
       </c>
       <c r="P42" s="13">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>9.2999999999999992E-3</v>
       </c>
       <c r="Q42" s="13">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1.24E-2</v>
       </c>
       <c r="R42" s="12"/>
@@ -3654,15 +3654,15 @@
         <v>8.4600000000000009E-2</v>
       </c>
       <c r="E43" s="8">
-        <f t="shared" si="7"/>
-        <v>971.11719411209049</v>
+        <f t="shared" si="9"/>
+        <v>1120.7835686544524</v>
       </c>
       <c r="F43" s="9">
         <v>0.3</v>
       </c>
       <c r="G43" s="10">
-        <f t="shared" si="8"/>
-        <v>22093.5</v>
+        <f t="shared" si="10"/>
+        <v>25498.5</v>
       </c>
       <c r="H43" s="11"/>
       <c r="I43" s="12"/>
@@ -3701,15 +3701,15 @@
         <v>0.10050000000000001</v>
       </c>
       <c r="E44" s="8">
-        <f t="shared" si="7"/>
-        <v>1730.0832808390956</v>
+        <f t="shared" si="9"/>
+        <v>1996.7197834872554</v>
       </c>
       <c r="F44" s="9">
         <v>0.6</v>
       </c>
       <c r="G44" s="10">
-        <f t="shared" si="8"/>
-        <v>44187</v>
+        <f t="shared" si="10"/>
+        <v>50997</v>
       </c>
       <c r="H44" s="11"/>
       <c r="I44" s="12"/>
@@ -3748,15 +3748,15 @@
         <v>9.2899999999999996E-2</v>
       </c>
       <c r="E45" s="8">
-        <f t="shared" si="7"/>
-        <v>1371.9039876116672</v>
+        <f t="shared" si="9"/>
+        <v>1583.3387117530538</v>
       </c>
       <c r="F45" s="9">
         <v>0.55000000000000004</v>
       </c>
       <c r="G45" s="10">
-        <f t="shared" si="8"/>
-        <v>40504.75</v>
+        <f t="shared" si="10"/>
+        <v>46747.250000000007</v>
       </c>
       <c r="H45" s="11"/>
       <c r="I45" s="20"/>
@@ -3795,26 +3795,26 @@
         <v>8.6199999999999999E-2</v>
       </c>
       <c r="E46" s="8">
-        <f t="shared" si="7"/>
-        <v>1174.2080427339276</v>
+        <f t="shared" si="9"/>
+        <v>1355.1743172268339</v>
       </c>
       <c r="F46" s="9">
         <v>0.5</v>
       </c>
       <c r="G46" s="10">
-        <f t="shared" si="8"/>
-        <v>36822.5</v>
+        <f t="shared" si="10"/>
+        <v>42497.5</v>
       </c>
       <c r="H46" s="11"/>
-      <c r="I46" s="29"/>
-      <c r="J46" s="29"/>
-      <c r="K46" s="29"/>
-      <c r="L46" s="29"/>
-      <c r="M46" s="29"/>
-      <c r="N46" s="29"/>
-      <c r="O46" s="29"/>
-      <c r="P46" s="29"/>
-      <c r="Q46" s="29"/>
+      <c r="I46" s="30"/>
+      <c r="J46" s="30"/>
+      <c r="K46" s="30"/>
+      <c r="L46" s="30"/>
+      <c r="M46" s="30"/>
+      <c r="N46" s="30"/>
+      <c r="O46" s="30"/>
+      <c r="P46" s="30"/>
+      <c r="Q46" s="30"/>
       <c r="R46" s="12"/>
       <c r="S46" s="12"/>
       <c r="T46" s="12"/>
@@ -3842,15 +3842,15 @@
         <v>9.1300000000000006E-2</v>
       </c>
       <c r="E47" s="8">
-        <f t="shared" si="7"/>
-        <v>1144.1661325104765</v>
+        <f>PMT(D47/12,C47,-84995,G47)</f>
+        <v>1320.5024160870114</v>
       </c>
       <c r="F47" s="9">
         <v>0.4</v>
       </c>
       <c r="G47" s="10">
-        <f t="shared" si="8"/>
-        <v>29458</v>
+        <f>SUM(84995*F47)</f>
+        <v>33998</v>
       </c>
       <c r="H47" s="11"/>
       <c r="I47" s="20"/>
@@ -4725,14 +4725,14 @@
         <v>7.3999999999999996E-2</v>
       </c>
       <c r="E66" s="8">
-        <f t="shared" ref="E66:E91" si="14">PMT(D66/12,C66,-dealTotal,G66)</f>
+        <f t="shared" ref="E66:E91" si="16">PMT(D66/12,C66,-dealTotal,G66)</f>
         <v>943.51795120806958</v>
       </c>
       <c r="F66" s="9">
         <v>0.4</v>
       </c>
       <c r="G66" s="10">
-        <f t="shared" ref="G66:G91" si="15">SUM(dealTotal*F66)</f>
+        <f t="shared" ref="G66:G91" si="17">SUM(dealTotal*F66)</f>
         <v>29458</v>
       </c>
       <c r="I66" s="12"/>
@@ -4771,14 +4771,14 @@
         <v>7.3599999999999999E-2</v>
       </c>
       <c r="E67" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>889.01988647834901</v>
       </c>
       <c r="F67" s="9">
         <v>0.35</v>
       </c>
       <c r="G67" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>25775.75</v>
       </c>
       <c r="I67" s="12"/>
@@ -4817,14 +4817,14 @@
         <v>9.0499999999999997E-2</v>
       </c>
       <c r="E68" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>1679.7006572197906</v>
       </c>
       <c r="F68" s="9">
         <v>0.6</v>
       </c>
       <c r="G68" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>44187</v>
       </c>
       <c r="I68" s="12"/>
@@ -4863,14 +4863,14 @@
         <v>8.6199999999999999E-2</v>
       </c>
       <c r="E69" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>1338.9589139262678</v>
       </c>
       <c r="F69" s="9">
         <v>0.55000000000000004</v>
       </c>
       <c r="G69" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>40504.75</v>
       </c>
       <c r="I69" s="12"/>
@@ -4909,14 +4909,14 @@
         <v>8.1100000000000005E-2</v>
       </c>
       <c r="E70" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>1149.7060765599892</v>
       </c>
       <c r="F70" s="9">
         <v>0.5</v>
       </c>
       <c r="G70" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>36822.5</v>
       </c>
       <c r="I70" s="12"/>
@@ -4955,14 +4955,14 @@
         <v>7.669999999999999E-2</v>
       </c>
       <c r="E71" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>1026.7296144058514</v>
       </c>
       <c r="F71" s="9">
         <v>0.45</v>
       </c>
       <c r="G71" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>33140.25</v>
       </c>
       <c r="I71" s="12"/>
@@ -5001,14 +5001,14 @@
         <v>7.3999999999999996E-2</v>
       </c>
       <c r="E72" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>943.51795120806958</v>
       </c>
       <c r="F72" s="9">
         <v>0.4</v>
       </c>
       <c r="G72" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>29458</v>
       </c>
       <c r="I72" s="12"/>
@@ -5047,14 +5047,14 @@
         <v>7.3599999999999999E-2</v>
       </c>
       <c r="E73" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>889.01988647834901</v>
       </c>
       <c r="F73" s="9">
         <v>0.35</v>
       </c>
       <c r="G73" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>25775.75</v>
       </c>
       <c r="I73" s="12"/>
@@ -5093,14 +5093,14 @@
         <v>0.10050000000000001</v>
       </c>
       <c r="E74" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>1730.0832808390956</v>
       </c>
       <c r="F74" s="9">
         <v>0.6</v>
       </c>
       <c r="G74" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>44187</v>
       </c>
       <c r="I74" s="12"/>
@@ -5139,14 +5139,14 @@
         <v>9.2899999999999996E-2</v>
       </c>
       <c r="E75" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>1371.9039876116672</v>
       </c>
       <c r="F75" s="9">
         <v>0.55000000000000004</v>
       </c>
       <c r="G75" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>40504.75</v>
       </c>
       <c r="I75" s="12"/>
@@ -5185,14 +5185,14 @@
         <v>8.6199999999999999E-2</v>
       </c>
       <c r="E76" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>1174.2080427339276</v>
       </c>
       <c r="F76" s="9">
         <v>0.5</v>
       </c>
       <c r="G76" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>36822.5</v>
       </c>
       <c r="I76" s="12"/>
@@ -5231,14 +5231,14 @@
         <v>8.09E-2</v>
       </c>
       <c r="E77" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>1046.4565539464597</v>
       </c>
       <c r="F77" s="9">
         <v>0.45</v>
       </c>
       <c r="G77" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>33140.25</v>
       </c>
       <c r="I77" s="12"/>
@@ -5277,14 +5277,14 @@
         <v>7.7499999999999999E-2</v>
       </c>
       <c r="E78" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>959.60817823346019</v>
       </c>
       <c r="F78" s="9">
         <v>0.4</v>
       </c>
       <c r="G78" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>29458</v>
       </c>
       <c r="I78" s="12"/>
@@ -5323,14 +5323,14 @@
         <v>7.669999999999999E-2</v>
       </c>
       <c r="E79" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>903.00454007282838</v>
       </c>
       <c r="F79" s="9">
         <v>0.35</v>
       </c>
       <c r="G79" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>25775.75</v>
       </c>
       <c r="I79" s="12"/>
@@ -5369,14 +5369,14 @@
         <v>0.1105</v>
       </c>
       <c r="E80" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>1780.5462518518855</v>
       </c>
       <c r="F80" s="9">
         <v>0.6</v>
       </c>
       <c r="G80" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>44187</v>
       </c>
       <c r="I80" s="12"/>
@@ -5415,14 +5415,14 @@
         <v>9.9599999999999994E-2</v>
       </c>
       <c r="E81" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>1404.9098171470985</v>
       </c>
       <c r="F81" s="9">
         <v>0.55000000000000004</v>
       </c>
       <c r="G81" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>40504.75</v>
       </c>
       <c r="I81" s="12"/>
@@ -5461,14 +5461,14 @@
         <v>9.1299999999999992E-2</v>
       </c>
       <c r="E82" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>1198.7620093421735</v>
       </c>
       <c r="F82" s="9">
         <v>0.5</v>
       </c>
       <c r="G82" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>36822.5</v>
       </c>
       <c r="I82" s="12"/>
@@ -5507,14 +5507,14 @@
         <v>8.5099999999999995E-2</v>
       </c>
       <c r="E83" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>1066.2318098759959</v>
       </c>
       <c r="F83" s="9">
         <v>0.45</v>
       </c>
       <c r="G83" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>33140.25</v>
       </c>
       <c r="I83" s="12"/>
@@ -5553,14 +5553,14 @@
         <v>8.0999999999999989E-2</v>
       </c>
       <c r="E84" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>975.7421230508603</v>
       </c>
       <c r="F84" s="9">
         <v>0.4</v>
       </c>
       <c r="G84" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>29458</v>
       </c>
       <c r="I84" s="12"/>
@@ -5599,14 +5599,14 @@
         <v>7.9799999999999996E-2</v>
       </c>
       <c r="E85" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>917.03223890887227</v>
       </c>
       <c r="F85" s="9">
         <v>0.35</v>
       </c>
       <c r="G85" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>25775.75</v>
       </c>
       <c r="I85" s="12"/>
@@ -5645,14 +5645,14 @@
         <v>0.1205</v>
       </c>
       <c r="E86" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>1831.0894040326464</v>
       </c>
       <c r="F86" s="9">
         <v>0.6</v>
       </c>
       <c r="G86" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>44187</v>
       </c>
       <c r="I86" s="12"/>
@@ -5691,14 +5691,14 @@
         <v>0.10630000000000001</v>
       </c>
       <c r="E87" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>1437.9762826152451</v>
       </c>
       <c r="F87" s="9">
         <v>0.55000000000000004</v>
       </c>
       <c r="G87" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>40504.75</v>
       </c>
       <c r="I87" s="12"/>
@@ -5737,14 +5737,14 @@
         <v>9.64E-2</v>
       </c>
       <c r="E88" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>1223.3678692864696</v>
       </c>
       <c r="F88" s="9">
         <v>0.5</v>
       </c>
       <c r="G88" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>36822.5</v>
       </c>
       <c r="I88" s="12"/>
@@ -5789,7 +5789,7 @@
         <v>0.45</v>
       </c>
       <c r="G89" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>33140.25</v>
       </c>
       <c r="I89" s="12"/>
@@ -5828,14 +5828,14 @@
         <v>8.4499999999999992E-2</v>
       </c>
       <c r="E90" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>991.91968070898156</v>
       </c>
       <c r="F90" s="9">
         <v>0.4</v>
       </c>
       <c r="G90" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>29458</v>
       </c>
       <c r="I90" s="12"/>
@@ -5874,14 +5874,14 @@
         <v>8.2899999999999988E-2</v>
       </c>
       <c r="E91" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>931.10286581611911</v>
       </c>
       <c r="F91" s="9">
         <v>0.35</v>
       </c>
       <c r="G91" s="10">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>25775.75</v>
       </c>
       <c r="I91" s="12"/>
@@ -5920,7 +5920,7 @@
         <v>9.2999999999999999E-2</v>
       </c>
       <c r="E92" s="8">
-        <f t="shared" ref="E92:E121" si="16">PMT(D92/12,C92,-dealTotal)</f>
+        <f t="shared" ref="E92:E121" si="18">PMT(D92/12,C92,-dealTotal)</f>
         <v>3374.5988042124136</v>
       </c>
       <c r="F92" s="9"/>
@@ -5961,7 +5961,7 @@
         <v>8.8700000000000001E-2</v>
       </c>
       <c r="E93" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>2337.4380632947859</v>
       </c>
       <c r="F93" s="9"/>
@@ -6002,7 +6002,7 @@
         <v>8.6199999999999999E-2</v>
       </c>
       <c r="E94" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1819.399502134522</v>
       </c>
       <c r="F94" s="9"/>
@@ -6043,7 +6043,7 @@
         <v>8.4699999999999998E-2</v>
       </c>
       <c r="E95" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1509.8753494347279</v>
       </c>
       <c r="F95" s="9"/>
@@ -6084,7 +6084,7 @@
         <v>8.4000000000000005E-2</v>
       </c>
       <c r="E96" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1305.6665582350709</v>
       </c>
       <c r="F96" s="9"/>
@@ -6104,7 +6104,7 @@
         <v>8.3600000000000008E-2</v>
       </c>
       <c r="E97" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1161.0999609661169</v>
       </c>
       <c r="F97" s="9"/>
@@ -6124,7 +6124,7 @@
         <v>9.2999999999999999E-2</v>
       </c>
       <c r="E98" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>3374.5988042124136</v>
       </c>
       <c r="F98" s="9"/>
@@ -6144,7 +6144,7 @@
         <v>8.8700000000000001E-2</v>
       </c>
       <c r="E99" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>2337.4380632947859</v>
       </c>
       <c r="F99" s="9"/>
@@ -6164,7 +6164,7 @@
         <v>8.6199999999999999E-2</v>
       </c>
       <c r="E100" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1819.399502134522</v>
       </c>
       <c r="F100" s="9"/>
@@ -6184,7 +6184,7 @@
         <v>8.4699999999999998E-2</v>
       </c>
       <c r="E101" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1509.8753494347279</v>
       </c>
       <c r="F101" s="9"/>
@@ -6204,7 +6204,7 @@
         <v>8.4000000000000005E-2</v>
       </c>
       <c r="E102" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1305.6665582350709</v>
       </c>
       <c r="F102" s="9"/>
@@ -6224,7 +6224,7 @@
         <v>8.3600000000000008E-2</v>
       </c>
       <c r="E103" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1161.0999609661169</v>
       </c>
       <c r="F103" s="9"/>
@@ -6244,7 +6244,7 @@
         <v>0.10300000000000001</v>
       </c>
       <c r="E104" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>3408.5493685450183</v>
       </c>
       <c r="F104" s="9"/>
@@ -6264,7 +6264,7 @@
         <v>9.5399999999999999E-2</v>
       </c>
       <c r="E105" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>2360.4438531486621</v>
       </c>
       <c r="F105" s="9"/>
@@ -6284,7 +6284,7 @@
         <v>9.1300000000000006E-2</v>
       </c>
       <c r="E106" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1837.2083103510142</v>
       </c>
       <c r="F106" s="9"/>
@@ -6304,7 +6304,7 @@
         <v>8.8900000000000007E-2</v>
       </c>
       <c r="E107" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1524.820422490707</v>
       </c>
       <c r="F107" s="9"/>
@@ -6324,7 +6324,7 @@
         <v>8.7500000000000008E-2</v>
       </c>
       <c r="E108" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1318.371453694388</v>
       </c>
       <c r="F108" s="9"/>
@@ -6344,7 +6344,7 @@
         <v>8.6699999999999999E-2</v>
       </c>
       <c r="E109" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1172.5835731738177</v>
       </c>
       <c r="F109" s="9"/>
@@ -6364,7 +6364,7 @@
         <v>0.113</v>
       </c>
       <c r="E110" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>3442.7006988330681</v>
       </c>
       <c r="F110" s="9"/>
@@ -6384,7 +6384,7 @@
         <v>0.1021</v>
       </c>
       <c r="E111" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>2383.5845577385107</v>
       </c>
       <c r="F111" s="9"/>
@@ -6404,7 +6404,7 @@
         <v>9.6400000000000013E-2</v>
       </c>
       <c r="E112" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1855.1209052396057</v>
       </c>
       <c r="F112" s="9"/>
@@ -6424,7 +6424,7 @@
         <v>9.3100000000000002E-2</v>
       </c>
       <c r="E113" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1539.8529629640348</v>
       </c>
       <c r="F113" s="9"/>
@@ -6444,7 +6444,7 @@
         <v>9.0999999999999998E-2</v>
       </c>
       <c r="E114" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1331.1486971491438</v>
       </c>
       <c r="F114" s="9"/>
@@ -6464,7 +6464,7 @@
         <v>8.9800000000000005E-2</v>
       </c>
       <c r="E115" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1184.1328077713738</v>
       </c>
       <c r="F115" s="9"/>
@@ -6484,7 +6484,7 @@
         <v>0.123</v>
       </c>
       <c r="E116" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>3477.0523758862673</v>
       </c>
       <c r="F116" s="9"/>
@@ -6504,7 +6504,7 @@
         <v>0.10880000000000001</v>
       </c>
       <c r="E117" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>2406.8599068564636</v>
       </c>
       <c r="F117" s="9"/>
@@ -6524,7 +6524,7 @@
         <v>0.10150000000000001</v>
       </c>
       <c r="E118" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1873.1370647111671</v>
       </c>
       <c r="F118" s="9"/>
@@ -6544,7 +6544,7 @@
         <v>9.7299999999999998E-2</v>
       </c>
       <c r="E119" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1554.9727609258252</v>
       </c>
       <c r="F119" s="9"/>
@@ -6564,7 +6564,7 @@
         <v>9.4500000000000001E-2</v>
       </c>
       <c r="E120" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1343.998097393385</v>
       </c>
       <c r="F120" s="9"/>
@@ -6584,7 +6584,7 @@
         <v>9.2899999999999996E-2</v>
       </c>
       <c r="E121" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>1195.7474670564322</v>
       </c>
       <c r="F121" s="9"/>
@@ -7387,17 +7387,17 @@
         <v>25775.75</v>
       </c>
       <c r="H12" s="11"/>
-      <c r="I12" s="30" t="s">
+      <c r="I12" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="J12" s="30"/>
-      <c r="K12" s="30"/>
-      <c r="L12" s="30"/>
-      <c r="M12" s="30"/>
-      <c r="N12" s="30"/>
-      <c r="O12" s="30"/>
-      <c r="P12" s="30"/>
-      <c r="Q12" s="30"/>
+      <c r="J12" s="29"/>
+      <c r="K12" s="29"/>
+      <c r="L12" s="29"/>
+      <c r="M12" s="29"/>
+      <c r="N12" s="29"/>
+      <c r="O12" s="29"/>
+      <c r="P12" s="29"/>
+      <c r="Q12" s="29"/>
       <c r="R12" s="11"/>
       <c r="S12" s="11"/>
       <c r="T12" s="11"/>

</xml_diff>